<commit_message>
Usunięte słupki 22 kW: z obliczeń, raportu, Excela, oferty i cennika szablonu (wersja 1.43)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XygCrjT9K7zVw2zg8hs3qQ
</commit_message>
<xml_diff>
--- a/kalkulator-nk38/przyklady/Kalkulator_ul_Lesna_5_Wroclaw_NK41.xlsx
+++ b/kalkulator-nk38/przyklady/Kalkulator_ul_Lesna_5_Wroclaw_NK41.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="151">
   <si>
     <t>KALKULACJA NK41</t>
   </si>
@@ -42,7 +42,7 @@
     <t>21.10.2026</t>
   </si>
   <si>
-    <t>Wygenerowano 27.10.2026, 14:16:58 · ceny netto w zł · szablon NK41</t>
+    <t>Wygenerowano 27.10.2026, 14:20:07 · ceny netto w zł · szablon NK41</t>
   </si>
   <si>
     <t>Cena ofertowa · zysk 14%</t>
@@ -190,12 +190,6 @@
   </si>
   <si>
     <t>46 MP × 1700 zł + montaż</t>
-  </si>
-  <si>
-    <t>Słupki e-ładowarek 22 kW</t>
-  </si>
-  <si>
-    <t>jak 3,7 kW + 4600 zł/MP</t>
   </si>
   <si>
     <t>Konserwacja · wariant 1 · 23 szt.</t>
@@ -1305,7 +1299,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1816,79 +1810,75 @@
         <v>108853.26834744174</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="37" t="s">
+    <row r="41" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="38" t="s">
+      <c r="B41" s="40"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="C40" s="38"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="39">
-        <v>374029.1183359035</v>
-      </c>
-      <c r="F40" s="39">
-        <v>359550.0590451161</v>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="40" t="s">
+      <c r="E41" s="40"/>
+      <c r="F41" s="40"/>
+    </row>
+    <row r="42" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="B42" s="40"/>
-      <c r="C42" s="40"/>
-      <c r="D42" s="40" t="s">
+      <c r="B42" s="41"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="E42" s="40"/>
-      <c r="F42" s="40"/>
-    </row>
-    <row r="43" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="41" t="s">
+      <c r="E42" s="41"/>
+      <c r="F42" s="41"/>
+    </row>
+    <row r="43" ht="17" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="B43" s="41"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="41" t="s">
+      <c r="B43" s="42"/>
+      <c r="C43" s="42"/>
+      <c r="D43" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
-    </row>
-    <row r="44" ht="17" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="42" t="s">
+      <c r="E43" s="42"/>
+      <c r="F43" s="42"/>
+    </row>
+    <row r="44" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="B44" s="42"/>
-      <c r="C44" s="42"/>
-      <c r="D44" s="42" t="s">
+      <c r="B44" s="43"/>
+      <c r="C44" s="43"/>
+      <c r="D44" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="E44" s="42"/>
-      <c r="F44" s="42"/>
-    </row>
-    <row r="45" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="43" t="s">
+      <c r="E44" s="43"/>
+      <c r="F44" s="43"/>
+    </row>
+    <row r="46" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B45" s="43"/>
-      <c r="C45" s="43"/>
-      <c r="D45" s="43" t="s">
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
-    </row>
-    <row r="47" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="10" t="s">
+      <c r="B47" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
+      <c r="C47" s="45"/>
+      <c r="D47" s="45"/>
+      <c r="E47" s="45"/>
+      <c r="F47" s="45"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="44" t="s">
@@ -1926,20 +1916,8 @@
       <c r="E50" s="45"/>
       <c r="F50" s="45"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="B51" s="45" t="s">
-        <v>72</v>
-      </c>
-      <c r="C51" s="45"/>
-      <c r="D51" s="45"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-    </row>
   </sheetData>
-  <mergeCells count="59">
+  <mergeCells count="58">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:D2"/>
@@ -1985,20 +1963,19 @@
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="D41:F41"/>
     <mergeCell ref="A42:C42"/>
     <mergeCell ref="D42:F42"/>
     <mergeCell ref="A43:C43"/>
     <mergeCell ref="D43:F43"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="D44:F44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="B47:F47"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B51:F51"/>
   </mergeCells>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.25" footer="0.25"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="80" fitToWidth="1" fitToHeight="1"/>
@@ -2019,7 +1996,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -2028,7 +2005,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -2037,7 +2014,7 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -2046,10 +2023,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="44" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B5" s="45" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="45"/>
@@ -2057,10 +2034,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="44" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C6" s="45"/>
       <c r="D6" s="45"/>
@@ -2068,10 +2045,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="44" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B7" s="45" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C7" s="45"/>
       <c r="D7" s="45"/>
@@ -2079,10 +2056,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="44" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C8" s="45"/>
       <c r="D8" s="45"/>
@@ -2090,10 +2067,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="44" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C9" s="45"/>
       <c r="D9" s="45"/>
@@ -2101,10 +2078,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="44" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C10" s="45"/>
       <c r="D10" s="45"/>
@@ -2112,10 +2089,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="44" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="45"/>
@@ -2123,7 +2100,7 @@
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -2132,23 +2109,23 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="47" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B14" s="47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C14" s="47"/>
       <c r="D14" s="47"/>
       <c r="E14" s="48" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="49" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B15" s="50" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C15" s="50"/>
       <c r="D15" s="50"/>
@@ -2158,10 +2135,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="52" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C16" s="53"/>
       <c r="D16" s="53"/>
@@ -2171,10 +2148,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="49" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B17" s="50" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C17" s="50"/>
       <c r="D17" s="50"/>
@@ -2184,10 +2161,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="52" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C18" s="53"/>
       <c r="D18" s="53"/>
@@ -2197,10 +2174,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="49" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B19" s="50" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="50"/>
@@ -2210,10 +2187,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="52" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B20" s="53" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C20" s="53"/>
       <c r="D20" s="53"/>
@@ -2226,7 +2203,7 @@
         <v>22</v>
       </c>
       <c r="B21" s="50" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C21" s="50"/>
       <c r="D21" s="50"/>
@@ -2236,10 +2213,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="52" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B22" s="53" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C22" s="53"/>
       <c r="D22" s="53"/>
@@ -2249,10 +2226,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="49" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B23" s="50" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C23" s="50"/>
       <c r="D23" s="50"/>
@@ -2265,7 +2242,7 @@
         <v>41</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C24" s="53"/>
       <c r="D24" s="53"/>
@@ -2275,10 +2252,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="49" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B25" s="50" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C25" s="50"/>
       <c r="D25" s="50"/>
@@ -2288,10 +2265,10 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="52" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B26" s="53" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C26" s="53"/>
       <c r="D26" s="53"/>
@@ -2301,10 +2278,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="49" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B27" s="50" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C27" s="50"/>
       <c r="D27" s="50"/>
@@ -2314,10 +2291,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="52" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B28" s="53" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C28" s="53"/>
       <c r="D28" s="53"/>
@@ -2330,7 +2307,7 @@
         <v>40</v>
       </c>
       <c r="B29" s="50" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C29" s="50"/>
       <c r="D29" s="50"/>
@@ -2340,10 +2317,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="52" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B30" s="53" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C30" s="53"/>
       <c r="D30" s="53"/>
@@ -2353,10 +2330,10 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="58" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B31" s="59" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C31" s="59"/>
       <c r="D31" s="59"/>
@@ -2366,10 +2343,10 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="52" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B32" s="53" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C32" s="53"/>
       <c r="D32" s="53"/>
@@ -2379,10 +2356,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="49" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B33" s="50" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C33" s="50"/>
       <c r="D33" s="50"/>
@@ -2392,10 +2369,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="52" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B34" s="53" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C34" s="53"/>
       <c r="D34" s="53"/>
@@ -2405,10 +2382,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="49" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B35" s="50" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C35" s="50"/>
       <c r="D35" s="50"/>
@@ -2418,10 +2395,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="52" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B36" s="53" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C36" s="53"/>
       <c r="D36" s="53"/>
@@ -2431,10 +2408,10 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="58" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B37" s="59" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C37" s="59"/>
       <c r="D37" s="59"/>
@@ -2444,10 +2421,10 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="58" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B38" s="59" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C38" s="59"/>
       <c r="D38" s="59"/>
@@ -2457,7 +2434,7 @@
     </row>
     <row r="39" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="46" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B39" s="46"/>
       <c r="C39" s="46"/>
@@ -2466,7 +2443,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
@@ -2481,67 +2458,67 @@
         <v>34</v>
       </c>
       <c r="C42" s="63" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D42" s="63"/>
       <c r="E42" s="64" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="43" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="63" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B43" s="65">
         <v>130</v>
       </c>
       <c r="C43" s="63" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D43" s="63"/>
       <c r="E43" s="64" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="63" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B44" s="65">
         <v>45</v>
       </c>
       <c r="C44" s="63" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D44" s="63"/>
       <c r="E44" s="64" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="45" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="61" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B45" s="62" t="s">
         <v>34</v>
       </c>
       <c r="C45" s="63" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D45" s="63"/>
       <c r="E45" s="64" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="46" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="63" t="s">
+        <v>145</v>
+      </c>
+      <c r="B46" s="64" t="s">
+        <v>146</v>
+      </c>
+      <c r="C46" s="61" t="s">
         <v>147</v>
-      </c>
-      <c r="B46" s="64" t="s">
-        <v>148</v>
-      </c>
-      <c r="C46" s="61" t="s">
-        <v>149</v>
       </c>
       <c r="D46" s="61"/>
       <c r="E46" s="62" t="s">
@@ -2550,17 +2527,17 @@
     </row>
     <row r="47" ht="13" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="61" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B47" s="62" t="s">
         <v>34</v>
       </c>
       <c r="C47" s="63" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D47" s="63"/>
       <c r="E47" s="64" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>